<commit_message>
Treat the DV01 band as dollars plus dust, and check KR01 node by node.
The ±2% limit is unchanged. Endpoints at $49,000 and $51,000 per bp now pass. Published P&L and the five book decisions do not move.
</commit_message>
<xml_diff>
--- a/fixed_income_case.xlsx
+++ b/fixed_income_case.xlsx
@@ -1860,23 +1860,23 @@
         <v>49</v>
       </c>
       <c r="B17" s="0" t="str">
-        <f aca="false">IF(ABS(B15/DV01Target-1)&lt;=0.02,"inside","outside")</f>
+        <f aca="false">IF(ABS(B15-DV01Target)&lt;=DV01Target*0.02+0.000001,"inside","outside")</f>
         <v>inside</v>
       </c>
       <c r="C17" s="0" t="str">
-        <f aca="false">IF(ABS(C15/DV01Target-1)&lt;=0.02,"inside","outside")</f>
+        <f aca="false">IF(ABS(C15-DV01Target)&lt;=DV01Target*0.02+0.000001,"inside","outside")</f>
         <v>inside</v>
       </c>
       <c r="D17" s="0" t="str">
-        <f aca="false">IF(ABS(D15/DV01Target-1)&lt;=0.02,"inside","outside")</f>
+        <f aca="false">IF(ABS(D15-DV01Target)&lt;=DV01Target*0.02+0.000001,"inside","outside")</f>
         <v>inside</v>
       </c>
       <c r="E17" s="0" t="str">
-        <f aca="false">IF(ABS(E15/DV01Target-1)&lt;=0.02,"inside","outside")</f>
+        <f aca="false">IF(ABS(E15-DV01Target)&lt;=DV01Target*0.02+0.000001,"inside","outside")</f>
         <v>inside</v>
       </c>
       <c r="F17" s="0" t="str">
-        <f aca="false">IF(ABS(F15/DV01Target-1)&lt;=0.02,"inside","outside")</f>
+        <f aca="false">IF(ABS(F15-DV01Target)&lt;=DV01Target*0.02+0.000001,"inside","outside")</f>
         <v>inside</v>
       </c>
     </row>
@@ -2560,23 +2560,23 @@
         <v>81</v>
       </c>
       <c r="B49" s="13" t="b">
-        <f aca="false">ABS(B15/DV01Target-1)&lt;=0.02</f>
+        <f aca="false">ABS(B15-DV01Target)&lt;=DV01Target*0.02+0.000001</f>
         <v>1</v>
       </c>
       <c r="C49" s="13" t="b">
-        <f aca="false">ABS(C15/DV01Target-1)&lt;=0.02</f>
+        <f aca="false">ABS(C15-DV01Target)&lt;=DV01Target*0.02+0.000001</f>
         <v>1</v>
       </c>
       <c r="D49" s="13" t="b">
-        <f aca="false">ABS(D15/DV01Target-1)&lt;=0.02</f>
+        <f aca="false">ABS(D15-DV01Target)&lt;=DV01Target*0.02+0.000001</f>
         <v>1</v>
       </c>
       <c r="E49" s="13" t="b">
-        <f aca="false">ABS(E15/DV01Target-1)&lt;=0.02</f>
+        <f aca="false">ABS(E15-DV01Target)&lt;=DV01Target*0.02+0.000001</f>
         <v>1</v>
       </c>
       <c r="F49" s="13" t="b">
-        <f aca="false">ABS(F15/DV01Target-1)&lt;=0.02</f>
+        <f aca="false">ABS(F15-DV01Target)&lt;=DV01Target*0.02+0.000001</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>